<commit_message>
Add class answers + LTSS definition to Oct 30 sign-ups sheet
</commit_message>
<xml_diff>
--- a/assets/Oct30-Class-Signups-and-Questions-2026-10-26.xlsx
+++ b/assets/Oct30-Class-Signups-and-Questions-2026-10-26.xlsx
@@ -490,7 +490,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J8"/>
+  <dimension ref="A1:K8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -503,6 +503,7 @@
     <col width="22" customWidth="1" min="8" max="8"/>
     <col width="62" customWidth="1" min="9" max="9"/>
     <col width="42" customWidth="1" min="10" max="10"/>
+    <col width="105" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -570,8 +571,13 @@
           <t>What They Hope to Learn</t>
         </is>
       </c>
-    </row>
-    <row r="4" ht="62" customHeight="1">
+      <c r="K3" s="3" t="inlineStr">
+        <is>
+          <t>Answer — Ready to Say in Class (plain words)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="285" customHeight="1">
       <c r="A4" s="4" t="n">
         <v>1</v>
       </c>
@@ -620,8 +626,17 @@
           <t>When they are a DAC, can they pay rent from their third party trust, or only from their ABLE? Thank you.</t>
         </is>
       </c>
-    </row>
-    <row r="5" ht="62" customHeight="1">
+      <c r="K4" s="9" t="inlineStr">
+        <is>
+          <t>WHAT LTSS IS: LTSS = Long-Term Services and Supports — the ongoing help Texas Medicaid gives a person with a disability to live day to day: a helper (attendant) at home for bathing, dressing and meals, respite (a break for the family caregiver), day programs, and help in a group home or host home. It usually comes through the Texas waiver programs: CLASS, HCS, TxHmL, and STAR+PLUS. LTSS is Medicaid help — it is NOT the Social Security check.
+Q1 — Opt out of LTSS, stay a DAC? YES, she can stay a DAC.
+DAC is her monthly check from Social Security. LTSS is help from Texas Medicaid. They are not the same thing. If she stops LTSS, her DAC check does NOT stop. Warn first: the LTSS help stops too, she may lose her spot and wait a long time to get it back, and her Medicaid might change — check with Texas (HHSC / her MCO, in writing) before she stops.
+Q2 — Rent from trust or only ABLE? Rent can be paid from BOTH.
+ABLE: best if she still gets SSI — rent from ABLE does NOT cut SSI if the money is taken out and paid in the same month. Trust: the trustee can pay the landlord directly (do not hand her cash for rent). If she still gets SSI, her SSI goes down a little (not all). If she gets only DAC and no SSI, trust-paid rent does NOT cut her DAC check.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="235" customHeight="1">
       <c r="A5" s="6" t="n">
         <v>2</v>
       </c>
@@ -666,8 +681,15 @@
         </is>
       </c>
       <c r="J5" s="7" t="inlineStr"/>
-    </row>
-    <row r="6" ht="62" customHeight="1">
+      <c r="K5" s="9" t="inlineStr">
+        <is>
+          <t>Not by itself. SSI does not give her the other one. They are 2 different programs.
+SSI is help for people with very low money — no work history needed. Social Security disability is based on work — her own work, or a parent's work (called DAC). For DAC: her disability must have started before age 22; her parent must have worked and paid in; her parent must be retired, disabled, or have passed away. Her age now is 33 — that does NOT stop her; what counts is when her disability started. If she gets DAC, her SSI may go down or stop, but she can often keep Medicaid. After 2 years on DAC, she can get Medicare. Social Security must look and decide.
+En español: Recibir SSI no significa que también recibirá el otro pago. Son dos programas diferentes. Ella puede calificar en el récord de un padre si su discapacidad comenzó antes de los 22 años, y el padre ya está jubilado, discapacitado, o falleció. Tener 33 años ahora no la detiene. El Seguro Social tiene que revisar su caso y decidir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="265" customHeight="1">
       <c r="A6" s="4" t="n">
         <v>3</v>
       </c>
@@ -716,8 +738,17 @@
           <t>yes all of my options for support and what I can do in the future</t>
         </is>
       </c>
-    </row>
-    <row r="7" ht="62" customHeight="1">
+      <c r="K6" s="9" t="inlineStr">
+        <is>
+          <t>Child support counts for SSI — but Social Security does NOT count all of it.
+It counts as the child's own money (unearned income), and only what she actually got that month counts. First Social Security leaves out one-third (1/3) of the child support, then leaves out $20 more. Only what is left lowers the SSI check, dollar for dollar. Example: $300 support → leave out $100 → leave out $20 → $180 counts → SSI goes down $180 that month.
+Only the parent the child lives with has their pay counted — the other parent's job pay does NOT count, only the support actually paid. Her own work pay can count too, but SSA first sets aside money for her to live on and an amount for her other child.
+For her 4-year-old: a clear diagnosis is step one — SSI needs medical papers showing the diagnosis and daily limits. Two free doors: her doctor can refer for a full evaluation, and the school district must do a free evaluation when a parent asks in writing (Child Find, ages 3–21).
+Options: SSI brings Medicaid in Texas; SNAP (food help); 2-1-1 Texas; a free first talk after class to map her family's numbers. Warn: tell SSA when support starts, stops, or changes — unreported changes cause overpayments.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
       <c r="A7" s="6" t="n">
         <v>4</v>
       </c>
@@ -766,8 +797,13 @@
           <t>(nothing written)</t>
         </is>
       </c>
-    </row>
-    <row r="8" ht="62" customHeight="1">
+      <c r="K7" s="9" t="inlineStr">
+        <is>
+          <t>(No question submitted — nothing to answer.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="430" customHeight="1">
       <c r="A8" s="4" t="n">
         <v>5</v>
       </c>
@@ -814,6 +850,14 @@
       <c r="J8" s="5" t="inlineStr">
         <is>
           <t>All of it. 😉thank you</t>
+        </is>
+      </c>
+      <c r="K8" s="9" t="inlineStr">
+        <is>
+          <t>Q1 — Should my son be receiving DAC? He may be — and your own disability may be the key.
+DAC is a check for an adult child on a parent's work record: he is 18 or older; his disability started before age 22 (when it started counts, not his age now); he is not married (a few exceptions); and a parent is retired, receiving disability, or has passed away. If you receive Social Security disability (SSDI), that is exactly the parent record a son can be paid DAC on — he does not need his own work history. DAC does not start by itself — someone has to ask Social Security to check and file. If DAC starts and his SSI goes down or stops, Medicaid can often stay, and Medicare can follow after 24 months on DAC. Say plainly: "I can't decide this in class — Social Security has to look at his records and decide in writing. But this is worth asking them about, by name: DAC."
+Q2 — Can I do his CLASS hours and not affect my disability? Do NOT give a yes/no in class — it depends on facts we don't have. CLASS is a Texas Medicaid waiver, not Social Security. If the hours are UNPAID family help: not wages, so they do not count as earnings against her disability check (but SSA can ask about work-like activity at a medical review — keep it honest). If the hours are ever PAID (for example through Consumer Directed Services, CDS): pay IS wages — it counts toward SSDI work limits (Trial Work Period / substantial gainful activity) or lowers an SSI check, and must be counted BEFORE she starts. Texas CLASS rules allow pay to a parent/legal guardian of a person over 17 for some services (residential habilitation and respite), not for routine family care — details sit with her son's CLASS case manager / HHSC, in writing. Safe class line: "Paid or unpaid changes the answer, and so does which disability check you get. Don't start paid hours until we run your numbers — that's a one-on-one talk after class."
+Q3 — ABLE vs. trust, with and without an LLC: Both protect benefits; they do different jobs, and an LLC does not change the Social Security rules. ABLE: the person with the disability controls it; good for everyday costs and rent — rent from ABLE does not cut SSI if taken out and paid in the same month; yearly deposit limit; first $100,000 does not count against SSI. Third-party trust: no yearly limit, better for larger amounts and inheritances, and no Medicaid payback at the end; if the trustee pays rent directly and the person still gets SSI, SSI goes down a little (it does not cut a DAC-only check). The LLC part: Social Security looks at who owns the money, who controls it, and whether her son can get cash or shelter from it — not the wrapper's name. An LLC does not by itself make it safe or unsafe; that set-up needs a Texas special-needs attorney before any money moves. Safe class line: "Many families use both — ABLE for rent and everyday costs, a trust for the bigger money."</t>
         </is>
       </c>
     </row>
@@ -834,7 +878,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A10"/>
+  <dimension ref="A1:A13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -898,6 +942,20 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Answers added Mon Oct 26, 2026: column K holds the plain-words answer for every question (7 questions, 4 families). Full combined sheet: Oct30-Class-QA-ALL-Families-Combined-2026-10-26.md in your_files.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>LTSS = Long-Term Services and Supports — Texas Medicaid’s ongoing help for a person with a disability (home attendant, respite, day programs; waivers CLASS, HCS, TxHmL, STAR+PLUS). Not a Social Security check. Definition also added at the top of Linda’s answer in column K (Oct 26, 2026).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>